<commit_message>
Docs: Help names both daily limits and the practice look; rules sheet v2.1; deploy order with db push; what this chat built
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F27FTLtQrEqPZa6zkJZdvH
</commit_message>
<xml_diff>
--- a/docs/srs-review-plan-rules.xlsx
+++ b/docs/srs-review-plan-rules.xlsx
@@ -81,12 +81,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="218">
   <si>
     <t xml:space="preserve">Spaced Repetition · Your Review Plan — rules for review</t>
   </si>
   <si>
-    <t xml:space="preserve">Version 2.0 · 30 Oct 2026 · the rules as built in spaced repetition v2 (docs/SRS-V2-PLAN.md). Version 1.0 had the old rules (1 · 3 · 7 · 15 · 30 · 60 days).</t>
+    <t xml:space="preserve">Version 2.1 · 30 Oct 2026 · the rules as built in spaced repetition v2, with the fixes from both audits (docs/SRS-V2-PLAN.md). Version 1.0 had the old rules (1 · 3 · 7 · 15 · 30 · 60 days).</t>
   </si>
   <si>
     <t xml:space="preserve">What this file is</t>
@@ -341,7 +341,7 @@
     <t xml:space="preserve">R12</t>
   </si>
   <si>
-    <t xml:space="preserve">After Unknown, the card comes round once more in the same session, 3 cards later, marked 'Practice · not saved'. That answer only moves on; nothing is saved. If nothing else is left, it comes at once.</t>
+    <t xml:space="preserve">After Unknown, the card comes round once more in the same session, 3 cards later, with the line 'Practice · not saved. Cards you mark Unknown come round once more like this.' That answer only moves on; nothing is saved and the date does not change. If nothing else is left, it comes at once.</t>
   </si>
   <si>
     <t xml:space="preserve">Once, after 3 cards</t>
@@ -437,7 +437,7 @@
     <t xml:space="preserve">R19</t>
   </si>
   <si>
-    <t xml:space="preserve">Reviews per day (Settings): No limit, 50, 100, 150 or 200, per kind (Words, Chunks, Grammar, Support) per India day. Past the limit, due cards wait for tomorrow and new cards are still served.</t>
+    <t xml:space="preserve">Reviews per day (Settings): No limit, 50, 100, 150 or 200, per kind (Words, Chunks, Grammar, Support) per India day. Past the limit, due cards wait for tomorrow and new cards are still served. A review is an answer today on a card first answered on an earlier day.</t>
   </si>
   <si>
     <t xml:space="preserve">Default = No limit</t>
@@ -473,6 +473,21 @@
     <t xml:space="preserve">10 chunks done → no new idioms today either</t>
   </si>
   <si>
+    <t xml:space="preserve">R21b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New or review is decided by the card's first answer (saved once, firstReviewedAt), not by when a remark was added and not by how many answers it has. A card tagged yesterday and first answered today is new; a new card opened again with ‹ and answered again the same day is still one new card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First answer decides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tag Mon, first answer Tue → new on Tue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/flashcards.ts, lib/todayReview.ts</t>
+  </si>
+  <si>
     <t xml:space="preserve">R22</t>
   </si>
   <si>
@@ -491,7 +506,7 @@
     <t xml:space="preserve">R23</t>
   </si>
   <si>
-    <t xml:space="preserve">Due counts on the Flashcard tab, Today page and Dashboard stop at the review limit, so they match what today will serve.</t>
+    <t xml:space="preserve">Due counts on the Flashcard tab, Today page, Dashboard and the reminder email stop at the review limit, so they match what today will serve.</t>
   </si>
   <si>
     <t xml:space="preserve">Capped</t>
@@ -500,7 +515,7 @@
     <t xml:space="preserve">140 due, limit 100 → shows 100</t>
   </si>
   <si>
-    <t xml:space="preserve">lib/todayReview.ts</t>
+    <t xml:space="preserve">lib/srs.ts (servableDue)</t>
   </si>
   <si>
     <t xml:space="preserve">R24</t>
@@ -584,10 +599,13 @@
     <t xml:space="preserve">R31</t>
   </si>
   <si>
-    <t xml:space="preserve">The daily email reminder (if the student turned it on) is sent at their chosen hour, only when built-in cards are due.</t>
+    <t xml:space="preserve">The daily email reminder (if the student turned it on) is sent at their chosen hour, only when built-in cards are due. The number in it stops at the student's review limit; when the limit is used up, no email.</t>
   </si>
   <si>
     <t xml:space="preserve">Only if cards due</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limit 50, 45 done, 10 due → '5 flashcards are due'</t>
   </si>
   <si>
     <t xml:space="preserve">lib/studyReminders.ts</t>
@@ -1455,7 +1473,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -1777,7 +1795,7 @@
       <c r="H14" s="18"/>
       <c r="I14" s="18"/>
     </row>
-    <row r="15" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
         <v>85</v>
       </c>
@@ -1964,7 +1982,7 @@
       <c r="H23" s="18"/>
       <c r="I23" s="18"/>
     </row>
-    <row r="24" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
         <v>117</v>
       </c>
@@ -2033,12 +2051,12 @@
       <c r="H26" s="18"/>
       <c r="I26" s="18"/>
     </row>
-    <row r="27" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
         <v>130</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>131</v>
@@ -2056,12 +2074,12 @@
       <c r="H27" s="18"/>
       <c r="I27" s="18"/>
     </row>
-    <row r="28" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
         <v>135</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="C28" s="16" t="s">
         <v>136</v>
@@ -2083,8 +2101,8 @@
       <c r="A29" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="B29" s="8" t="s">
-        <v>61</v>
+      <c r="B29" s="15" t="s">
+        <v>51</v>
       </c>
       <c r="C29" s="16" t="s">
         <v>141</v>
@@ -2093,164 +2111,164 @@
         <v>142</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>40</v>
+        <v>143</v>
       </c>
       <c r="F29" s="17" t="s">
-        <v>116</v>
+        <v>144</v>
       </c>
       <c r="G29" s="5"/>
       <c r="H29" s="18"/>
       <c r="I29" s="18"/>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
-      <c r="I30" s="13"/>
-    </row>
-    <row r="31" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="B31" s="8" t="s">
+    <row r="30" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B30" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C31" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="D31" s="16" t="s">
+      <c r="C30" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="E31" s="16" t="s">
+      <c r="D30" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="E30" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="F31" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="G31" s="5"/>
-      <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="s">
+      <c r="F30" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="G30" s="5"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="13"/>
-    </row>
-    <row r="33" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14" t="s">
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="13"/>
+    </row>
+    <row r="32" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B32" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C33" s="16" t="s">
+      <c r="C32" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="D33" s="16" t="s">
+      <c r="D32" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="E33" s="16" t="s">
+      <c r="E32" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="F33" s="17" t="s">
+      <c r="F32" s="17" t="s">
         <v>152</v>
       </c>
-      <c r="G33" s="5"/>
-      <c r="H33" s="18"/>
-      <c r="I33" s="18"/>
-    </row>
-    <row r="34" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G32" s="5"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="18"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="13"/>
+      <c r="G33" s="13"/>
+      <c r="H33" s="13"/>
+      <c r="I33" s="13"/>
+    </row>
+    <row r="34" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B34" s="8" t="s">
         <v>61</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="E34" s="16" t="s">
         <v>40</v>
       </c>
       <c r="F34" s="17" t="s">
-        <v>107</v>
+        <v>157</v>
       </c>
       <c r="G34" s="5"/>
       <c r="H34" s="18"/>
       <c r="I34" s="18"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B35" s="13"/>
-      <c r="C35" s="13"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="13"/>
-    </row>
-    <row r="36" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="14" t="s">
+    <row r="35" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="D35" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="B36" s="15" t="s">
+      <c r="E35" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="G35" s="5"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="18"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
+      <c r="G36" s="13"/>
+      <c r="H36" s="13"/>
+      <c r="I36" s="13"/>
+    </row>
+    <row r="37" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="B37" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C36" s="16" t="s">
-        <v>157</v>
-      </c>
-      <c r="D36" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="E36" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="F36" s="17" t="s">
-        <v>159</v>
-      </c>
-      <c r="G36" s="5"/>
-      <c r="H36" s="18"/>
-      <c r="I36" s="18"/>
-    </row>
-    <row r="37" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>61</v>
-      </c>
       <c r="C37" s="16" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D37" s="16" t="s">
         <v>40</v>
       </c>
       <c r="E37" s="16" t="s">
-        <v>40</v>
+        <v>163</v>
       </c>
       <c r="F37" s="17" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="G37" s="5"/>
       <c r="H37" s="18"/>
@@ -2258,13 +2276,13 @@
     </row>
     <row r="38" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="14" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B38" s="8" t="s">
         <v>61</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D38" s="16" t="s">
         <v>40</v>
@@ -2279,94 +2297,104 @@
       <c r="H38" s="18"/>
       <c r="I38" s="18"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="13"/>
-      <c r="H39" s="13"/>
-      <c r="I39" s="13"/>
-    </row>
-    <row r="40" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="14" t="s">
-        <v>166</v>
-      </c>
-      <c r="B40" s="8" t="s">
+    <row r="39" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="B39" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C40" s="16" t="s">
-        <v>167</v>
-      </c>
-      <c r="D40" s="16" t="s">
+      <c r="C39" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="E40" s="16" t="s">
+      <c r="D39" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="F40" s="17" t="s">
+      <c r="E39" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="F39" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="G40" s="5"/>
-      <c r="H40" s="18"/>
-      <c r="I40" s="18"/>
-    </row>
-    <row r="41" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G39" s="5"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="18"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="13"/>
+      <c r="F40" s="13"/>
+      <c r="G40" s="13"/>
+      <c r="H40" s="13"/>
+      <c r="I40" s="13"/>
+    </row>
+    <row r="41" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>61</v>
+        <v>171</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>37</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>40</v>
+        <v>173</v>
       </c>
       <c r="E41" s="16" t="s">
-        <v>40</v>
+        <v>174</v>
       </c>
       <c r="F41" s="17" t="s">
-        <v>107</v>
+        <v>175</v>
       </c>
       <c r="G41" s="5"/>
       <c r="H41" s="18"/>
       <c r="I41" s="18"/>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="B42" s="13"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
-      <c r="F42" s="13"/>
-      <c r="G42" s="13"/>
-      <c r="H42" s="13"/>
-      <c r="I42" s="13"/>
-    </row>
-    <row r="43" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="B43" s="18"/>
-      <c r="C43" s="18"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
-      <c r="F43" s="18"/>
-      <c r="G43" s="5"/>
-      <c r="H43" s="18"/>
-      <c r="I43" s="18"/>
+    <row r="42" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C42" s="16" t="s">
+        <v>177</v>
+      </c>
+      <c r="D42" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="E42" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="F42" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="G42" s="5"/>
+      <c r="H42" s="18"/>
+      <c r="I42" s="18"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="B43" s="13"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="13"/>
+      <c r="F43" s="13"/>
+      <c r="G43" s="13"/>
+      <c r="H43" s="13"/>
+      <c r="I43" s="13"/>
     </row>
     <row r="44" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="14" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="B44" s="18"/>
       <c r="C44" s="18"/>
@@ -2379,7 +2407,7 @@
     </row>
     <row r="45" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="14" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B45" s="18"/>
       <c r="C45" s="18"/>
@@ -2392,7 +2420,7 @@
     </row>
     <row r="46" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="14" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B46" s="18"/>
       <c r="C46" s="18"/>
@@ -2405,7 +2433,7 @@
     </row>
     <row r="47" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="14" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B47" s="18"/>
       <c r="C47" s="18"/>
@@ -2416,20 +2444,33 @@
       <c r="H47" s="18"/>
       <c r="I47" s="18"/>
     </row>
+    <row r="48" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="B48" s="18"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="18"/>
+      <c r="E48" s="18"/>
+      <c r="F48" s="18"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="18"/>
+      <c r="I48" s="18"/>
+    </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="A16:I16"/>
     <mergeCell ref="A21:I21"/>
-    <mergeCell ref="A30:I30"/>
-    <mergeCell ref="A32:I32"/>
-    <mergeCell ref="A35:I35"/>
-    <mergeCell ref="A39:I39"/>
-    <mergeCell ref="A42:I42"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A33:I33"/>
+    <mergeCell ref="A36:I36"/>
+    <mergeCell ref="A40:I40"/>
+    <mergeCell ref="A43:I43"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" prompt="Pick Keep, Change, Remove or Not sure" promptTitle="Keep or change?" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G3:G6 G8:G15 G17:G20 G22:G29 G31 G33:G34 G36:G38 G40:G41 G43:G47" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" prompt="Pick Keep, Change, Remove or Not sure" promptTitle="Keep or change?" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G3:G6 G8:G15 G17:G20 G22:G30 G32 G34:G35 G37:G39 G41:G42 G44:G48" type="list">
       <formula1>"Keep,Change,Remove,Not sure"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2467,12 +2508,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -2487,18 +2528,18 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2512,7 +2553,7 @@
         <v>3</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2590,23 +2631,23 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>17</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="B17" s="9" t="n">
         <v>0</v>
@@ -2615,12 +2656,12 @@
         <v>0</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B18" s="9" t="n">
         <v>1</v>
@@ -2629,12 +2670,12 @@
         <v>1</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="21" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B19" s="9" t="n">
         <v>2</v>
@@ -2643,12 +2684,12 @@
         <v>2</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="21" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="B20" s="9" t="n">
         <v>2</v>
@@ -2657,12 +2698,12 @@
         <v>2</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="21" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="B21" s="9" t="n">
         <v>1</v>
@@ -2671,12 +2712,12 @@
         <v>1</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="21" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">COUNT(B6:B13)</f>
@@ -2687,44 +2728,44 @@
         <v>7</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="I25" s="12" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="J25" s="12" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="K25" s="12" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2732,7 +2773,7 @@
         <v>1</v>
       </c>
       <c r="B26" s="22" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C26" s="23" t="n">
         <f aca="false">IF(B26="","",IF(B26=$A$20,MAX(1,$B$21-$B$20),MAX(1,MIN($B$22,$B$21+VLOOKUP(B26,$A$17:$B$19,2,FALSE())))))</f>
@@ -2772,7 +2813,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="22" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C27" s="23" t="n">
         <f aca="false">IF(OR(B27="",C26=""),"",IF(B27=$A$20,MAX(1,C26-$B$20),MAX(1,MIN($B$22,C26+VLOOKUP(B27,$A$17:$B$19,2,FALSE())))))</f>
@@ -2812,7 +2853,7 @@
         <v>3</v>
       </c>
       <c r="B28" s="22" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="C28" s="23" t="n">
         <f aca="false">IF(OR(B28="",C27=""),"",IF(B28=$A$20,MAX(1,C27-$B$20),MAX(1,MIN($B$22,C27+VLOOKUP(B28,$A$17:$B$19,2,FALSE())))))</f>
@@ -2852,7 +2893,7 @@
         <v>4</v>
       </c>
       <c r="B29" s="22" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C29" s="23" t="n">
         <f aca="false">IF(OR(B29="",C28=""),"",IF(B29=$A$20,MAX(1,C28-$B$20),MAX(1,MIN($B$22,C28+VLOOKUP(B29,$A$17:$B$19,2,FALSE())))))</f>
@@ -2892,7 +2933,7 @@
         <v>5</v>
       </c>
       <c r="B30" s="22" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C30" s="23" t="n">
         <f aca="false">IF(OR(B30="",C29=""),"",IF(B30=$A$20,MAX(1,C29-$B$20),MAX(1,MIN($B$22,C29+VLOOKUP(B30,$A$17:$B$19,2,FALSE())))))</f>
@@ -2932,7 +2973,7 @@
         <v>6</v>
       </c>
       <c r="B31" s="22" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C31" s="23" t="n">
         <f aca="false">IF(OR(B31="",C30=""),"",IF(B31=$A$20,MAX(1,C30-$B$20),MAX(1,MIN($B$22,C30+VLOOKUP(B31,$A$17:$B$19,2,FALSE())))))</f>
@@ -2972,7 +3013,7 @@
         <v>7</v>
       </c>
       <c r="B32" s="22" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C32" s="23" t="n">
         <f aca="false">IF(OR(B32="",C31=""),"",IF(B32=$A$20,MAX(1,C31-$B$20),MAX(1,MIN($B$22,C31+VLOOKUP(B32,$A$17:$B$19,2,FALSE())))))</f>
@@ -3012,7 +3053,7 @@
         <v>8</v>
       </c>
       <c r="B33" s="22" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C33" s="23" t="n">
         <f aca="false">IF(OR(B33="",C32=""),"",IF(B33=$A$20,MAX(1,C32-$B$20),MAX(1,MIN($B$22,C32+VLOOKUP(B33,$A$17:$B$19,2,FALSE())))))</f>
@@ -3052,7 +3093,7 @@
         <v>9</v>
       </c>
       <c r="B34" s="22" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C34" s="23" t="n">
         <f aca="false">IF(OR(B34="",C33=""),"",IF(B34=$A$20,MAX(1,C33-$B$20),MAX(1,MIN($B$22,C33+VLOOKUP(B34,$A$17:$B$19,2,FALSE())))))</f>
@@ -3092,7 +3133,7 @@
         <v>10</v>
       </c>
       <c r="B35" s="22" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C35" s="23" t="n">
         <f aca="false">IF(OR(B35="",C34=""),"",IF(B35=$A$20,MAX(1,C34-$B$20),MAX(1,MIN($B$22,C34+VLOOKUP(B35,$A$17:$B$19,2,FALSE())))))</f>
@@ -3132,7 +3173,7 @@
         <v>11</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C36" s="23" t="n">
         <f aca="false">IF(OR(B36="",C35=""),"",IF(B36=$A$20,MAX(1,C35-$B$20),MAX(1,MIN($B$22,C35+VLOOKUP(B36,$A$17:$B$19,2,FALSE())))))</f>
@@ -3172,7 +3213,7 @@
         <v>12</v>
       </c>
       <c r="B37" s="22" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C37" s="23" t="n">
         <f aca="false">IF(OR(B37="",C36=""),"",IF(B37=$A$20,MAX(1,C36-$B$20),MAX(1,MIN($B$22,C36+VLOOKUP(B37,$A$17:$B$19,2,FALSE())))))</f>
@@ -3513,7 +3554,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="10" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E47" s="14" t="n">
         <f aca="false">COUNT(C26:C45)</f>
@@ -3526,7 +3567,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="10" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="E48" s="14" t="n">
         <f aca="false">MAX(E26:E45)</f>

</xml_diff>